<commit_message>
compress trained model into a .zip file
</commit_message>
<xml_diff>
--- a/outputs/bootstrapped_metrics.xlsx
+++ b/outputs/bootstrapped_metrics.xlsx
@@ -447,16 +447,16 @@
         <v>0.931095406360424</v>
       </c>
       <c r="C2">
-        <v>0.9310141342756182</v>
+        <v>0.9309169611307418</v>
       </c>
       <c r="D2">
-        <v>0.9098939929328622</v>
+        <v>0.9081272084805654</v>
       </c>
       <c r="E2">
-        <v>0.9505742049469964</v>
+        <v>0.9522968197879859</v>
       </c>
       <c r="F2">
-        <v>0.01059892270029471</v>
+        <v>0.01074704630271923</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
@@ -470,16 +470,16 @@
         <v>0.9588377723970944</v>
       </c>
       <c r="C3">
-        <v>0.9592163575823115</v>
+        <v>0.9585343425786571</v>
       </c>
       <c r="D3">
-        <v>0.9404366829117351</v>
+        <v>0.9374890734265734</v>
       </c>
       <c r="E3">
-        <v>0.9775657363943083</v>
+        <v>0.9765258215962441</v>
       </c>
       <c r="F3">
-        <v>0.009577762832778895</v>
+        <v>0.01027751664629169</v>
       </c>
       <c r="G3" t="s">
         <v>12</v>
@@ -493,16 +493,16 @@
         <v>0.9473684210526315</v>
       </c>
       <c r="C4">
-        <v>0.9471583029541004</v>
+        <v>0.9469334770112765</v>
       </c>
       <c r="D4">
-        <v>0.9245686010595158</v>
+        <v>0.923856109541506</v>
       </c>
       <c r="E4">
-        <v>0.9680609252300428</v>
+        <v>0.9684504127386145</v>
       </c>
       <c r="F4">
-        <v>0.01095979778606956</v>
+        <v>0.01108487956635322</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
@@ -516,16 +516,16 @@
         <v>0.9530685920577617</v>
       </c>
       <c r="C5">
-        <v>0.9529172273990451</v>
+        <v>0.953324350896259</v>
       </c>
       <c r="D5">
-        <v>0.9375726697253907</v>
+        <v>0.9377289377289377</v>
       </c>
       <c r="E5">
-        <v>0.9671176875704349</v>
+        <v>0.9679753116504977</v>
       </c>
       <c r="F5">
-        <v>0.007578525624065862</v>
+        <v>0.007701973112057738</v>
       </c>
       <c r="G5" t="s">
         <v>12</v>
@@ -539,16 +539,16 @@
         <v>0.8237289976852435</v>
       </c>
       <c r="C6">
-        <v>0.8253017728623548</v>
+        <v>0.8242039995584376</v>
       </c>
       <c r="D6">
-        <v>0.773606347423956</v>
+        <v>0.7681923331929517</v>
       </c>
       <c r="E6">
-        <v>0.8763044951926391</v>
+        <v>0.8739785916715112</v>
       </c>
       <c r="F6">
-        <v>0.02753014272121387</v>
+        <v>0.02760114906117863</v>
       </c>
       <c r="G6" t="s">
         <v>12</v>
@@ -562,16 +562,16 @@
         <v>0.9363957597173145</v>
       </c>
       <c r="C7">
-        <v>0.9366872791519433</v>
+        <v>0.9365724381625439</v>
       </c>
       <c r="D7">
-        <v>0.9169169611307421</v>
+        <v>0.9151943462897526</v>
       </c>
       <c r="E7">
-        <v>0.9558303886925795</v>
+        <v>0.9540636042402827</v>
       </c>
       <c r="F7">
-        <v>0.01037687348999866</v>
+        <v>0.01006478037356432</v>
       </c>
       <c r="G7" t="s">
         <v>12</v>
@@ -585,16 +585,16 @@
         <v>0.9661016949152542</v>
       </c>
       <c r="C8">
-        <v>0.9658492455650467</v>
+        <v>0.9656616838977153</v>
       </c>
       <c r="D8">
-        <v>0.9480978773584905</v>
+        <v>0.946208858378785</v>
       </c>
       <c r="E8">
-        <v>0.9815789318208673</v>
+        <v>0.9823243454698115</v>
       </c>
       <c r="F8">
-        <v>0.008809032575392992</v>
+        <v>0.009165305806493891</v>
       </c>
       <c r="G8" t="s">
         <v>12</v>
@@ -608,16 +608,16 @@
         <v>0.9477434679334917</v>
       </c>
       <c r="C9">
-        <v>0.9475482681884243</v>
+        <v>0.9481471296011853</v>
       </c>
       <c r="D9">
-        <v>0.9245272224860758</v>
+        <v>0.9261080899668938</v>
       </c>
       <c r="E9">
-        <v>0.9678182205193699</v>
+        <v>0.9685990338164251</v>
       </c>
       <c r="F9">
-        <v>0.01110028623898598</v>
+        <v>0.01093242487078628</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
@@ -631,16 +631,16 @@
         <v>0.9568345323741008</v>
       </c>
       <c r="C10">
-        <v>0.956603029903768</v>
+        <v>0.9564538640792555</v>
       </c>
       <c r="D10">
-        <v>0.9416056219169501</v>
+        <v>0.941884527901477</v>
       </c>
       <c r="E10">
-        <v>0.9702031397415688</v>
+        <v>0.9691961334633009</v>
       </c>
       <c r="F10">
-        <v>0.007334946613765919</v>
+        <v>0.007166058227864775</v>
       </c>
       <c r="G10" t="s">
         <v>12</v>
@@ -654,16 +654,16 @@
         <v>0.8366266803680021</v>
       </c>
       <c r="C11">
-        <v>0.838010097235963</v>
+        <v>0.8381675951999911</v>
       </c>
       <c r="D11">
-        <v>0.787465939310329</v>
+        <v>0.7846481060746805</v>
       </c>
       <c r="E11">
-        <v>0.8883684717804233</v>
+        <v>0.8872337689428313</v>
       </c>
       <c r="F11">
-        <v>0.02573214987429557</v>
+        <v>0.02618147075507667</v>
       </c>
       <c r="G11" t="s">
         <v>12</v>
@@ -677,16 +677,16 @@
         <v>0.9434628975265018</v>
       </c>
       <c r="C12">
-        <v>0.9434081272084803</v>
+        <v>0.9427367491166074</v>
       </c>
       <c r="D12">
         <v>0.9240282685512368</v>
       </c>
       <c r="E12">
-        <v>0.9628975265017667</v>
+        <v>0.9611307420494699</v>
       </c>
       <c r="F12">
-        <v>0.009752912470227146</v>
+        <v>0.009751958641688293</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
@@ -700,16 +700,16 @@
         <v>0.9782082324455206</v>
       </c>
       <c r="C13">
-        <v>0.9781052091172184</v>
+        <v>0.9778732889544228</v>
       </c>
       <c r="D13">
-        <v>0.9634146341463414</v>
+        <v>0.9632165551131069</v>
       </c>
       <c r="E13">
-        <v>0.9904317612212349</v>
+        <v>0.9904545944138006</v>
       </c>
       <c r="F13">
-        <v>0.007146579894720155</v>
+        <v>0.007203184423791874</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
@@ -723,16 +723,16 @@
         <v>0.9461358313817331</v>
       </c>
       <c r="C14">
-        <v>0.9467699976141104</v>
+        <v>0.9462515536167835</v>
       </c>
       <c r="D14">
-        <v>0.9239592933947773</v>
+        <v>0.9244817447565877</v>
       </c>
       <c r="E14">
-        <v>0.9671727521112766</v>
+        <v>0.967367864693446</v>
       </c>
       <c r="F14">
-        <v>0.01086874493536992</v>
+        <v>0.01105571258859877</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
@@ -746,16 +746,16 @@
         <v>0.9619047619047619</v>
       </c>
       <c r="C15">
-        <v>0.9617215181266492</v>
+        <v>0.9618985138223347</v>
       </c>
       <c r="D15">
-        <v>0.9486447576585647</v>
+        <v>0.947482425018889</v>
       </c>
       <c r="E15">
-        <v>0.9743619489559164</v>
+        <v>0.9746558345251338</v>
       </c>
       <c r="F15">
-        <v>0.00675053423162037</v>
+        <v>0.006853210371354481</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
@@ -769,16 +769,16 @@
         <v>0.8542156963678194</v>
       </c>
       <c r="C16">
-        <v>0.8540171200840755</v>
+        <v>0.8540860056496462</v>
       </c>
       <c r="D16">
-        <v>0.8022880713370878</v>
+        <v>0.8028896703539546</v>
       </c>
       <c r="E16">
-        <v>0.8992900256486532</v>
+        <v>0.8990957721995129</v>
       </c>
       <c r="F16">
-        <v>0.02472134474668539</v>
+        <v>0.02434650423562806</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
update the bootstrap results
</commit_message>
<xml_diff>
--- a/outputs/bootstrapped_metrics.xlsx
+++ b/outputs/bootstrapped_metrics.xlsx
@@ -475,20 +475,20 @@
         <v>0.931095406360424</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9317279151943459</v>
+        <v>0.9314982332155475</v>
       </c>
       <c r="D2" t="n">
-        <v>0.911660777385159</v>
+        <v>0.9098939929328622</v>
       </c>
       <c r="E2" t="n">
-        <v>0.950530035335689</v>
+        <v>0.9522968197879859</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01036815534495657</v>
+        <v>0.01060277011720281</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ensemble_voting_soft</t>
+          <t>single</t>
         </is>
       </c>
     </row>
@@ -502,20 +502,20 @@
         <v>0.9588377723970944</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9587417760447553</v>
+        <v>0.9587611247831244</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9393884096438841</v>
+        <v>0.9390121374618001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9767000887485154</v>
+        <v>0.9779411764705882</v>
       </c>
       <c r="F3" t="n">
-        <v>0.009830424616860374</v>
+        <v>0.01001488630708052</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ensemble_voting_soft</t>
+          <t>single</t>
         </is>
       </c>
     </row>
@@ -529,20 +529,20 @@
         <v>0.9473684210526315</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9478607580547507</v>
+        <v>0.946839631986035</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9240814378629789</v>
+        <v>0.9232671783365387</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9679071350762527</v>
+        <v>0.9665891010342084</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0108340118937133</v>
+        <v>0.01114676214890244</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ensemble_voting_soft</t>
+          <t>single</t>
         </is>
       </c>
     </row>
@@ -556,20 +556,20 @@
         <v>0.9530685920577617</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9531258016624511</v>
+        <v>0.9529989682926328</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9375764993880049</v>
+        <v>0.9372701340686508</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9672727272727273</v>
+        <v>0.9671951839169336</v>
       </c>
       <c r="F5" t="n">
-        <v>0.007497542311404406</v>
+        <v>0.007763520244732173</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ensemble_voting_soft</t>
+          <t>single</t>
         </is>
       </c>
     </row>
@@ -583,20 +583,20 @@
         <v>0.8237289976852435</v>
       </c>
       <c r="C6" t="n">
-        <v>0.823577803084973</v>
+        <v>0.823981799098384</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7677332107113082</v>
+        <v>0.7644815971002296</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8754582200741392</v>
+        <v>0.8749402768779185</v>
       </c>
       <c r="F6" t="n">
-        <v>0.02730390755020331</v>
+        <v>0.02748161347822248</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ensemble_voting_soft</t>
+          <t>single</t>
         </is>
       </c>
     </row>
@@ -610,16 +610,16 @@
         <v>0.9363957597173145</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9367985865724379</v>
+        <v>0.9365883392226146</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9169611307420494</v>
+        <v>0.9187279151943463</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9558745583038869</v>
+        <v>0.9558303886925795</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01015371132334517</v>
+        <v>0.01001583218360101</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -637,16 +637,16 @@
         <v>0.9661016949152542</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9662448501808526</v>
+        <v>0.9655737039543437</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9478436897146918</v>
+        <v>0.9462069730092526</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9828871676809499</v>
+        <v>0.9819156231365533</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008943096785708074</v>
+        <v>0.009105116335700627</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -664,16 +664,16 @@
         <v>0.9477434679334917</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9477000371056593</v>
+        <v>0.9477332193899426</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9254052573932092</v>
+        <v>0.9256556831284408</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9677437893956248</v>
+        <v>0.9683758305783772</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01074272931324109</v>
+        <v>0.0107022557214718</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -691,16 +691,16 @@
         <v>0.9568345323741008</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9566109911292695</v>
+        <v>0.9563693454771999</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9411727802789873</v>
+        <v>0.9424420181169553</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9706979922733892</v>
+        <v>0.9692761151985152</v>
       </c>
       <c r="F10" t="n">
-        <v>0.007430668674565321</v>
+        <v>0.006993323073435897</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -718,16 +718,16 @@
         <v>0.8366266803680021</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8365435059135072</v>
+        <v>0.8373501696448342</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7848609896817557</v>
+        <v>0.7853736797800686</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8876368379682745</v>
+        <v>0.8868662864795882</v>
       </c>
       <c r="F11" t="n">
-        <v>0.02630989883400122</v>
+        <v>0.02631144827431252</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
         <v>0.9434628975265018</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9439575971731446</v>
+        <v>0.9436378091872789</v>
       </c>
       <c r="D12" t="n">
         <v>0.9240282685512368</v>
@@ -754,7 +754,7 @@
         <v>0.9611307420494699</v>
       </c>
       <c r="F12" t="n">
-        <v>0.009455450086633675</v>
+        <v>0.009634921981248056</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -772,16 +772,16 @@
         <v>0.9782082324455206</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9784526951387689</v>
+        <v>0.9785947831236429</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9642814422419685</v>
+        <v>0.9635922330097088</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9923857868020305</v>
+        <v>0.9905665926748057</v>
       </c>
       <c r="F13" t="n">
-        <v>0.007107839392787371</v>
+        <v>0.007164874617114366</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -799,16 +799,16 @@
         <v>0.9461358313817331</v>
       </c>
       <c r="C14" t="n">
-        <v>0.946256897623583</v>
+        <v>0.9463244461041351</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9234472934472935</v>
+        <v>0.9243454001546166</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9675944636900179</v>
+        <v>0.9675192811721234</v>
       </c>
       <c r="F14" t="n">
-        <v>0.01120922477462064</v>
+        <v>0.01104846945533329</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -826,16 +826,16 @@
         <v>0.9619047619047619</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9615393782849875</v>
+        <v>0.9618956764769618</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9464720194647201</v>
+        <v>0.946468755563468</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9745310090307137</v>
+        <v>0.9750297265160524</v>
       </c>
       <c r="F15" t="n">
-        <v>0.007121960988547928</v>
+        <v>0.00687896506365436</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
         <v>0.8542156963678194</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8543219659820279</v>
+        <v>0.8540623894654689</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8036308181069302</v>
+        <v>0.8028342154823694</v>
       </c>
       <c r="E16" t="n">
-        <v>0.9009419893176425</v>
+        <v>0.9007771938487327</v>
       </c>
       <c r="F16" t="n">
-        <v>0.02530097344353104</v>
+        <v>0.0244603979486431</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>

</xml_diff>